<commit_message>
docs(tracker): RACE-001 DONE, CORE-003/TRACK-001 in progress
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Docs/ProgressTracker.xlsx
+++ b/Docs/ProgressTracker.xlsx
@@ -55,14 +55,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00F2F2F2"/>
+        <bgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
-        <bgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00FFEB9C"/>
+        <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
@@ -707,14 +707,14 @@
           <t>RACE</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>IN REVIEW</t>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>code-reviewer approved for merge (pass 2) at 7832d0a. test-engineer independent validation in progress -- NOT yet merged to main. Update this row to DONE once merged.</t>
+          <t>code-reviewer approved across 2 passes at 7832d0a. test-engineer independently confirmed 442/442 Smoke tests from a from-scratch rebuild. Merged to main at 2c41989.</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
           <t>A</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>IN PROGRESS (implementation dispatched)</t>
         </is>
       </c>
     </row>
@@ -1216,7 +1216,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1253,7 +1253,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1290,7 +1290,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1327,7 +1327,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1364,7 +1364,7 @@
           <t>B, C</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1401,7 +1401,7 @@
           <t>C</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>IN PROGRESS (implementation dispatched)</t>
         </is>
       </c>
     </row>
@@ -1475,7 +1475,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr">
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1512,9 +1512,9 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>IN REVIEW (approved, pending test-engineer + merge)</t>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1586,7 +1586,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G23" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1623,7 +1623,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
+      <c r="G24" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1660,7 +1660,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G25" s="5" t="inlineStr">
+      <c r="G25" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1697,7 +1697,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
+      <c r="G26" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1734,7 +1734,7 @@
           <t>B</t>
         </is>
       </c>
-      <c r="G27" s="5" t="inlineStr">
+      <c r="G27" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1771,7 +1771,7 @@
           <t>B, D</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1808,7 +1808,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1845,7 +1845,7 @@
           <t>F, G</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G30" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -1882,7 +1882,7 @@
           <t>F</t>
         </is>
       </c>
-      <c r="G31" s="5" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
@@ -2579,7 +2579,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>IN PROGRESS -- CORE-001, CORE-002 DONE; RACE-001 in review; rest OPEN</t>
+          <t>IN PROGRESS -- CORE-001, CORE-002, RACE-001 DONE; CORE-003, TRACK-001 in progress; rest OPEN</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>NOT STARTED</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): TEST-001, CORE-003, TRACK-001 DONE
All three merged and verified on main (5506dcf, 7596b9e, 5d44744).
Final combined Smoke run on main: 458/458 succeeded (2 with expected
in-test warnings from TRACK-001's failed-bake tests), 0 failed, 0
notRun, all 34 project suites green.
</commit_message>
<xml_diff>
--- a/Docs/ProgressTracker.xlsx
+++ b/Docs/ProgressTracker.xlsx
@@ -1144,7 +1144,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>DONE (merged 5506dcf)</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>IN PROGRESS (implementation dispatched)</t>
+          <t>DONE (merged 7596b9e)</t>
         </is>
       </c>
     </row>
@@ -1440,7 +1440,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>IN PROGRESS (implementation dispatched)</t>
+          <t>DONE (merged 5d44744)</t>
         </is>
       </c>
     </row>

</xml_diff>